<commit_message>
Updated Operation page content and js function for upload multiple OB file upload and Updated API calling function an added code for valid response parameter while API request faild in jsion format
</commit_message>
<xml_diff>
--- a/DOC/Operation Sequence.xlsx
+++ b/DOC/Operation Sequence.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>SeqNo</t>
   </si>
@@ -43,21 +43,6 @@
   </si>
   <si>
     <t>Product</t>
-  </si>
-  <si>
-    <t>Skill</t>
-  </si>
-  <si>
-    <t>Grade</t>
-  </si>
-  <si>
-    <t>Folder</t>
-  </si>
-  <si>
-    <t>Seamlength</t>
-  </si>
-  <si>
-    <t>Direct</t>
   </si>
 </sst>
 </file>
@@ -414,7 +399,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -422,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.28515625" style="1" customWidth="1"/>
@@ -433,14 +418,10 @@
     <col min="6" max="6" width="12" style="1" customWidth="1"/>
     <col min="7" max="7" width="8.7109375" style="6" customWidth="1"/>
     <col min="8" max="8" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="10" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="9.140625" style="1"/>
+    <col min="9" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -465,23 +446,8 @@
       <c r="H1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="3"/>
       <c r="C2" s="2"/>
@@ -490,13 +456,8 @@
       <c r="F2" s="2"/>
       <c r="G2" s="4"/>
       <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="3"/>
       <c r="C3" s="2"/>
@@ -505,13 +466,8 @@
       <c r="F3" s="2"/>
       <c r="G3" s="4"/>
       <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="3"/>
       <c r="C4" s="2"/>
@@ -520,13 +476,8 @@
       <c r="F4" s="2"/>
       <c r="G4" s="4"/>
       <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="3"/>
       <c r="C5" s="2"/>
@@ -535,13 +486,8 @@
       <c r="F5" s="2"/>
       <c r="G5" s="4"/>
       <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="3"/>
       <c r="C6" s="2"/>
@@ -550,13 +496,8 @@
       <c r="F6" s="2"/>
       <c r="G6" s="4"/>
       <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="3"/>
       <c r="C7" s="2"/>
@@ -565,13 +506,8 @@
       <c r="F7" s="2"/>
       <c r="G7" s="4"/>
       <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="3"/>
       <c r="C8" s="2"/>
@@ -580,13 +516,8 @@
       <c r="F8" s="2"/>
       <c r="G8" s="4"/>
       <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="3"/>
       <c r="C9" s="2"/>
@@ -595,13 +526,8 @@
       <c r="F9" s="2"/>
       <c r="G9" s="4"/>
       <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="3"/>
       <c r="C10" s="2"/>
@@ -610,13 +536,8 @@
       <c r="F10" s="2"/>
       <c r="G10" s="4"/>
       <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="3"/>
       <c r="C11" s="2"/>
@@ -625,13 +546,8 @@
       <c r="F11" s="2"/>
       <c r="G11" s="4"/>
       <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="3"/>
       <c r="C12" s="2"/>
@@ -640,13 +556,8 @@
       <c r="F12" s="2"/>
       <c r="G12" s="4"/>
       <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="3"/>
       <c r="C13" s="2"/>
@@ -655,13 +566,8 @@
       <c r="F13" s="2"/>
       <c r="G13" s="4"/>
       <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="3"/>
       <c r="C14" s="2"/>
@@ -670,13 +576,8 @@
       <c r="F14" s="2"/>
       <c r="G14" s="4"/>
       <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="3"/>
       <c r="C15" s="2"/>
@@ -685,13 +586,8 @@
       <c r="F15" s="2"/>
       <c r="G15" s="4"/>
       <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="3"/>
       <c r="C16" s="2"/>
@@ -700,13 +596,8 @@
       <c r="F16" s="2"/>
       <c r="G16" s="4"/>
       <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="3"/>
       <c r="C17" s="2"/>
@@ -715,13 +606,8 @@
       <c r="F17" s="2"/>
       <c r="G17" s="4"/>
       <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="3"/>
       <c r="C18" s="2"/>
@@ -730,13 +616,8 @@
       <c r="F18" s="2"/>
       <c r="G18" s="4"/>
       <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="3"/>
       <c r="C19" s="2"/>
@@ -745,13 +626,8 @@
       <c r="F19" s="2"/>
       <c r="G19" s="4"/>
       <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
-      <c r="L19" s="2"/>
-      <c r="M19" s="2"/>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="3"/>
       <c r="C20" s="2"/>
@@ -760,13 +636,8 @@
       <c r="F20" s="2"/>
       <c r="G20" s="4"/>
       <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-      <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="3"/>
       <c r="C21" s="2"/>
@@ -775,13 +646,8 @@
       <c r="F21" s="2"/>
       <c r="G21" s="4"/>
       <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-      <c r="L21" s="2"/>
-      <c r="M21" s="2"/>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" s="3"/>
       <c r="C22" s="2"/>
@@ -790,13 +656,8 @@
       <c r="F22" s="2"/>
       <c r="G22" s="4"/>
       <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" s="3"/>
       <c r="C23" s="2"/>
@@ -805,13 +666,8 @@
       <c r="F23" s="2"/>
       <c r="G23" s="4"/>
       <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="3"/>
       <c r="C24" s="2"/>
@@ -820,13 +676,8 @@
       <c r="F24" s="2"/>
       <c r="G24" s="4"/>
       <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="3"/>
       <c r="C25" s="2"/>
@@ -835,13 +686,8 @@
       <c r="F25" s="2"/>
       <c r="G25" s="4"/>
       <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="3"/>
       <c r="C26" s="2"/>
@@ -850,13 +696,8 @@
       <c r="F26" s="2"/>
       <c r="G26" s="4"/>
       <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="3"/>
       <c r="C27" s="2"/>
@@ -865,13 +706,8 @@
       <c r="F27" s="2"/>
       <c r="G27" s="4"/>
       <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
-      <c r="K27" s="2"/>
-      <c r="L27" s="2"/>
-      <c r="M27" s="2"/>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" s="3"/>
       <c r="C28" s="2"/>
@@ -880,13 +716,8 @@
       <c r="F28" s="2"/>
       <c r="G28" s="4"/>
       <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
-      <c r="L28" s="2"/>
-      <c r="M28" s="2"/>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="3"/>
       <c r="C29" s="2"/>
@@ -895,13 +726,8 @@
       <c r="F29" s="2"/>
       <c r="G29" s="4"/>
       <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
-      <c r="L29" s="2"/>
-      <c r="M29" s="2"/>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
       <c r="B30" s="3"/>
       <c r="C30" s="2"/>
@@ -910,13 +736,8 @@
       <c r="F30" s="2"/>
       <c r="G30" s="4"/>
       <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
-      <c r="K30" s="2"/>
-      <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="3"/>
       <c r="C31" s="2"/>
@@ -925,13 +746,8 @@
       <c r="F31" s="2"/>
       <c r="G31" s="4"/>
       <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
-      <c r="J31" s="2"/>
-      <c r="K31" s="2"/>
-      <c r="L31" s="2"/>
-      <c r="M31" s="2"/>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="3"/>
       <c r="C32" s="2"/>
@@ -940,13 +756,8 @@
       <c r="F32" s="2"/>
       <c r="G32" s="4"/>
       <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
-      <c r="K32" s="2"/>
-      <c r="L32" s="2"/>
-      <c r="M32" s="2"/>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="3"/>
       <c r="C33" s="2"/>
@@ -955,13 +766,8 @@
       <c r="F33" s="2"/>
       <c r="G33" s="4"/>
       <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
-      <c r="K33" s="2"/>
-      <c r="L33" s="2"/>
-      <c r="M33" s="2"/>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="3"/>
       <c r="C34" s="2"/>
@@ -970,13 +776,8 @@
       <c r="F34" s="2"/>
       <c r="G34" s="4"/>
       <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
-      <c r="J34" s="2"/>
-      <c r="K34" s="2"/>
-      <c r="L34" s="2"/>
-      <c r="M34" s="2"/>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="3"/>
       <c r="C35" s="2"/>
@@ -985,13 +786,8 @@
       <c r="F35" s="2"/>
       <c r="G35" s="4"/>
       <c r="H35" s="2"/>
-      <c r="I35" s="2"/>
-      <c r="J35" s="2"/>
-      <c r="K35" s="2"/>
-      <c r="L35" s="2"/>
-      <c r="M35" s="2"/>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="3"/>
       <c r="C36" s="2"/>
@@ -1000,13 +796,8 @@
       <c r="F36" s="2"/>
       <c r="G36" s="4"/>
       <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
-      <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
-      <c r="L36" s="2"/>
-      <c r="M36" s="2"/>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="3"/>
       <c r="C37" s="2"/>
@@ -1015,13 +806,8 @@
       <c r="F37" s="2"/>
       <c r="G37" s="4"/>
       <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
-      <c r="J37" s="2"/>
-      <c r="K37" s="2"/>
-      <c r="L37" s="2"/>
-      <c r="M37" s="2"/>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="3"/>
       <c r="C38" s="2"/>
@@ -1030,13 +816,8 @@
       <c r="F38" s="2"/>
       <c r="G38" s="4"/>
       <c r="H38" s="2"/>
-      <c r="I38" s="2"/>
-      <c r="J38" s="2"/>
-      <c r="K38" s="2"/>
-      <c r="L38" s="2"/>
-      <c r="M38" s="2"/>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
       <c r="B39" s="3"/>
       <c r="C39" s="2"/>
@@ -1045,13 +826,8 @@
       <c r="F39" s="2"/>
       <c r="G39" s="4"/>
       <c r="H39" s="2"/>
-      <c r="I39" s="2"/>
-      <c r="J39" s="2"/>
-      <c r="K39" s="2"/>
-      <c r="L39" s="2"/>
-      <c r="M39" s="2"/>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="3"/>
       <c r="C40" s="2"/>
@@ -1060,13 +836,8 @@
       <c r="F40" s="2"/>
       <c r="G40" s="4"/>
       <c r="H40" s="2"/>
-      <c r="I40" s="2"/>
-      <c r="J40" s="2"/>
-      <c r="K40" s="2"/>
-      <c r="L40" s="2"/>
-      <c r="M40" s="2"/>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="2"/>
       <c r="B41" s="3"/>
       <c r="C41" s="2"/>
@@ -1075,13 +846,8 @@
       <c r="F41" s="2"/>
       <c r="G41" s="4"/>
       <c r="H41" s="2"/>
-      <c r="I41" s="2"/>
-      <c r="J41" s="2"/>
-      <c r="K41" s="2"/>
-      <c r="L41" s="2"/>
-      <c r="M41" s="2"/>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
       <c r="B42" s="3"/>
       <c r="C42" s="2"/>
@@ -1090,13 +856,8 @@
       <c r="F42" s="2"/>
       <c r="G42" s="4"/>
       <c r="H42" s="2"/>
-      <c r="I42" s="2"/>
-      <c r="J42" s="2"/>
-      <c r="K42" s="2"/>
-      <c r="L42" s="2"/>
-      <c r="M42" s="2"/>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
       <c r="B43" s="3"/>
       <c r="C43" s="2"/>
@@ -1105,13 +866,8 @@
       <c r="F43" s="2"/>
       <c r="G43" s="4"/>
       <c r="H43" s="2"/>
-      <c r="I43" s="2"/>
-      <c r="J43" s="2"/>
-      <c r="K43" s="2"/>
-      <c r="L43" s="2"/>
-      <c r="M43" s="2"/>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
       <c r="B44" s="3"/>
       <c r="C44" s="2"/>
@@ -1120,13 +876,8 @@
       <c r="F44" s="2"/>
       <c r="G44" s="4"/>
       <c r="H44" s="2"/>
-      <c r="I44" s="2"/>
-      <c r="J44" s="2"/>
-      <c r="K44" s="2"/>
-      <c r="L44" s="2"/>
-      <c r="M44" s="2"/>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
       <c r="B45" s="3"/>
       <c r="C45" s="2"/>
@@ -1135,11 +886,6 @@
       <c r="F45" s="2"/>
       <c r="G45" s="4"/>
       <c r="H45" s="2"/>
-      <c r="I45" s="2"/>
-      <c r="J45" s="2"/>
-      <c r="K45" s="2"/>
-      <c r="L45" s="2"/>
-      <c r="M45" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>